<commit_message>
update code metrics diagrams
</commit_message>
<xml_diff>
--- a/Info/Grader Info/Code Metrics/Code Metrics.xlsx
+++ b/Info/Grader Info/Code Metrics/Code Metrics.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="20" documentId="8_{0F2A74BB-77C7-43EA-A394-E9910AC0038E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02CDCCB9-5DA3-4201-8169-40A706D827D0}"/>
+  <xr:revisionPtr revIDLastSave="34" documentId="8_{0F2A74BB-77C7-43EA-A394-E9910AC0038E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{384D0C9A-A11C-4CA6-BF46-8D072282F249}"/>
   <bookViews>
-    <workbookView xWindow="9960" yWindow="2430" windowWidth="22320" windowHeight="15690" xr2:uid="{9D78A614-EFF9-4209-B1FE-812CC6A57E97}"/>
+    <workbookView xWindow="6960" yWindow="2040" windowWidth="28800" windowHeight="15345" xr2:uid="{9D78A614-EFF9-4209-B1FE-812CC6A57E97}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -176,30 +176,48 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Main!$A$2:$A$3</c:f>
+              <c:f>Main!$A$2:$A$6</c:f>
               <c:numCache>
                 <c:formatCode>m/d/yyyy</c:formatCode>
-                <c:ptCount val="2"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>46068</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>46074</c:v>
                 </c:pt>
+                <c:pt idx="2">
+                  <c:v>46083</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>46089</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>46094</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Main!$B$2:$B$3</c:f>
+              <c:f>Main!$B$2:$B$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>307</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>552</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>866</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1249</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1252</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -978,6 +996,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1295,7 +1317,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5883AF6-B31E-4FDF-929F-78787CBA5424}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="10.125" bestFit="1" customWidth="1"/>
@@ -1346,6 +1368,48 @@
         <v>2510</v>
       </c>
     </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="1">
+        <v>46083</v>
+      </c>
+      <c r="B4">
+        <v>866</v>
+      </c>
+      <c r="C4">
+        <v>172</v>
+      </c>
+      <c r="D4">
+        <v>3984</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="1">
+        <v>46089</v>
+      </c>
+      <c r="B5">
+        <v>1249</v>
+      </c>
+      <c r="C5">
+        <v>180</v>
+      </c>
+      <c r="D5">
+        <v>4943</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="1">
+        <v>46094</v>
+      </c>
+      <c r="B6">
+        <v>1252</v>
+      </c>
+      <c r="C6">
+        <v>209</v>
+      </c>
+      <c r="D6">
+        <v>5394</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
code metrics, burndown charts
</commit_message>
<xml_diff>
--- a/Info/Grader Info/Code Metrics/Code Metrics.xlsx
+++ b/Info/Grader Info/Code Metrics/Code Metrics.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="47" documentId="8_{0F2A74BB-77C7-43EA-A394-E9910AC0038E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{19168485-1F09-45E7-B318-4B601862995C}"/>
+  <xr:revisionPtr revIDLastSave="55" documentId="8_{0F2A74BB-77C7-43EA-A394-E9910AC0038E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{347A2329-A8B2-4D50-888F-73D98A4AB232}"/>
   <bookViews>
     <workbookView xWindow="10545" yWindow="900" windowWidth="24495" windowHeight="18495" xr2:uid="{9D78A614-EFF9-4209-B1FE-812CC6A57E97}"/>
   </bookViews>
@@ -1014,10 +1014,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1335,7 +1331,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5883AF6-B31E-4FDF-929F-78787CBA5424}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="10.125" bestFit="1" customWidth="1"/>
@@ -1470,6 +1466,34 @@
         <v>6686</v>
       </c>
     </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="1">
+        <v>46137</v>
+      </c>
+      <c r="B10">
+        <v>1728</v>
+      </c>
+      <c r="C10">
+        <v>256</v>
+      </c>
+      <c r="D10">
+        <v>6555</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="1">
+        <v>46139</v>
+      </c>
+      <c r="B11">
+        <v>2148</v>
+      </c>
+      <c r="C11">
+        <v>309</v>
+      </c>
+      <c r="D11">
+        <v>8544</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>